<commit_message>
docs(qms): refer to the 2025 pilot customer generically in the evidence pack
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/qms/evidence-2026/00_Overview_and_Map/EM26-00_Evidence_Map_2025_to_2026.xlsx
+++ b/docs/qms/evidence-2026/00_Overview_and_Map/EM26-00_Evidence_Map_2025_to_2026.xlsx
@@ -480,7 +480,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Audit package for the GSU appliance project</t>
+          <t>Audit package for the 2025 university pilot appliance project</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -667,7 +667,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>1. AJACE EchoMind AI LLM Appliance – Privacy, Security &amp; Compliance Overview for Grambling State University.docx</t>
+          <t>1. AJACE EchoMind AI LLM Appliance – Privacy, Security &amp; Compliance Overview for &lt;university pilot customer&gt;.docx</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">

</xml_diff>

<commit_message>
docs(qms): current GitHub evidence — v1.4.1 tag and the defect-fix commit
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/qms/evidence-2026/00_Overview_and_Map/EM26-00_Evidence_Map_2025_to_2026.xlsx
+++ b/docs/qms/evidence-2026/00_Overview_and_Map/EM26-00_Evidence_Map_2025_to_2026.xlsx
@@ -1659,7 +1659,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D59"/>
+  <dimension ref="A1:D61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -2966,6 +2966,50 @@
         </is>
       </c>
     </row>
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>SCR-18</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>github tag v1.4.1</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t>Screens/SCR-18_github_tag_v1.4.1.png</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="inlineStr">
+        <is>
+          <t>Screenshot 2026-10-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>SCR-19</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>github fix commit e0ed4d0</t>
+        </is>
+      </c>
+      <c r="C61" s="2" t="inlineStr">
+        <is>
+          <t>Screens/SCR-19_github_fix_commit_e0ed4d0.png</t>
+        </is>
+      </c>
+      <c r="D61" s="2" t="inlineStr">
+        <is>
+          <t>Screenshot 2026-10-06</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
docs(qms): project board evidence — 65 tracked tickets replace the 2025 Jira screens
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/qms/evidence-2026/00_Overview_and_Map/EM26-00_Evidence_Map_2025_to_2026.xlsx
+++ b/docs/qms/evidence-2026/00_Overview_and_Map/EM26-00_Evidence_Map_2025_to_2026.xlsx
@@ -1482,17 +1482,17 @@
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>15_Testing test cases + EM26-13; GitHub board (to populate)</t>
+          <t>GitHub issues #4–#68 on the project board + 15_Testing test cases + EM26-13 (SCR-20, SCR-21)</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Created</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>No Jira for the rebuilt product</t>
+          <t>GitHub issues replace Jira for the rebuilt product</t>
         </is>
       </c>
     </row>
@@ -1514,15 +1514,19 @@
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>EM26-12 + SCR-11 commit history; GitHub board (to populate)</t>
+          <t>GitHub project board (SCR-20) + EM26-12 + SCR-11 commit history</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>Partial</t>
-        </is>
-      </c>
-      <c r="F35" s="2" t="inlineStr"/>
+          <t>Created</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>Board created 2026-10-06; earlier work transcribed</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -1638,12 +1642,12 @@
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>GitHub board (to populate)</t>
+          <t>Screens/SCR-20_github_project_board.png</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Created</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr"/>
@@ -1659,7 +1663,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D61"/>
+  <dimension ref="A1:D63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -3010,6 +3014,50 @@
         </is>
       </c>
     </row>
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>SCR-20</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>github project board</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>Screens/SCR-20_github_project_board.png</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="inlineStr">
+        <is>
+          <t>Screenshot 2026-10-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>SCR-21</t>
+        </is>
+      </c>
+      <c r="B63" s="2" t="inlineStr">
+        <is>
+          <t>github defect ticket NC-2026-012</t>
+        </is>
+      </c>
+      <c r="C63" s="2" t="inlineStr">
+        <is>
+          <t>Screens/SCR-21_github_defect_ticket_NC-2026-012.png</t>
+        </is>
+      </c>
+      <c r="D63" s="2" t="inlineStr">
+        <is>
+          <t>Screenshot 2026-10-06</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
docs(qms): revision 1.1 approved (AR-2026-002) — review and NFR evidence signed off
Alexander Peter (review), Sheryl Nazareth (QA) and Anita Johan (Managing Director)
confirmed revision 1.1 on 2026-10-10. Approval record:
docs/qms/records/approvals/2026-10-10_AR-2026-002_revision_approval.md

- EM26-17 and EM26-18 rev 1.1: status APPROVED, signatures dated 2026-10-10
- EM26-00, EM26-12, EM26-16, EM26-16b rev 1.1 under the same approval
- REG-10, REG-01 and QM-01 point to AR-2026-002
- Client names stay out of the public copy (Client A–D)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/qms/evidence-2026/00_Overview_and_Map/EM26-00_Evidence_Map_2025_to_2026.xlsx
+++ b/docs/qms/evidence-2026/00_Overview_and_Map/EM26-00_Evidence_Map_2025_to_2026.xlsx
@@ -2262,7 +2262,7 @@
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>APPROVED — 2026-10-07 (AR-2026-001)</t>
+          <t>APPROVED — rev 1.1 2026-10-10 (AR-2026-002); rev 1.0 2026-10-07 (AR-2026-001)</t>
         </is>
       </c>
     </row>
@@ -2328,7 +2328,7 @@
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>APPROVED — 2026-10-07 (AR-2026-001)</t>
+          <t>APPROVED — rev 1.1 2026-10-10 (AR-2026-002); rev 1.0 2026-10-07 (AR-2026-001)</t>
         </is>
       </c>
     </row>
@@ -2350,7 +2350,7 @@
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>APPROVED — 2026-10-07 (AR-2026-001)</t>
+          <t>APPROVED — rev 1.1 2026-10-10 (AR-2026-002); rev 1.0 2026-10-07 (AR-2026-001)</t>
         </is>
       </c>
     </row>
@@ -2482,7 +2482,7 @@
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>APPROVED — 2026-10-07 (AR-2026-001)</t>
+          <t>APPROVED — rev 1.1 2026-10-10 (AR-2026-002); rev 1.0 2026-10-07 (AR-2026-001)</t>
         </is>
       </c>
     </row>

</xml_diff>